<commit_message>
Corrected reversed thresholds for uniformity_SNV_read_position system metric
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/system_level_metrics.xlsx
+++ b/profiles/human-primary-snv/system_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C72640B-C382-499B-A50D-2D2B6236A913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92F3912-330D-46B8-AB2D-C8370C58B601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -1181,13 +1181,13 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
1. Renamed uniformity_SNV_position system metric to uniformity_SNV_genome_position 2. Renamed uniformity_SNV_spacing system metric to uniformity_SNV_nearest_neighbour
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/system_level_metrics.xlsx
+++ b/profiles/human-primary-snv/system_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92F3912-330D-46B8-AB2D-C8370C58B601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB355C9-39CA-41F1-8D1E-F7ECBEA7BA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -80,12 +80,6 @@
     <t>Batch</t>
   </si>
   <si>
-    <t>uniformity_SNV_position</t>
-  </si>
-  <si>
-    <t>uniformity_SNV_spacing</t>
-  </si>
-  <si>
     <t>external_concordance_trinuc_context</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t>Percentage of somatic SNVs that overlap with gnomAD</t>
+  </si>
+  <si>
+    <t>uniformity_SNV_genome_position</t>
+  </si>
+  <si>
+    <t>uniformity_SNV_nearest_neighbour</t>
   </si>
 </sst>
 </file>
@@ -1096,10 +1096,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1123,18 +1123,18 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1158,18 +1158,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1193,18 +1193,18 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1228,18 +1228,18 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1263,18 +1263,18 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="K6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1298,18 +1298,18 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1333,18 +1333,18 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1364,10 +1364,10 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated references to somatic variant rate with somatic variant burden
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/system_level_metrics.xlsx
+++ b/profiles/human-primary-snv/system_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB355C9-39CA-41F1-8D1E-F7ECBEA7BA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B43ED9-BACF-4A48-923A-52E82374E14E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <t>cross_reactivity_gnomAD_overlap</t>
   </si>
   <si>
-    <t>snv_rate.value</t>
-  </si>
-  <si>
     <t>percent_gnomAD_overlap.value</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
     <t>EX.MET_TRINUC_SIMILARITIES</t>
   </si>
   <si>
-    <t>EX.MET_SOMATIC_VARIANT_RATE</t>
-  </si>
-  <si>
     <t>Percentage of somatic SNVs that are called in &gt;1 sample</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t>uniformity_SNV_nearest_neighbour</t>
+  </si>
+  <si>
+    <t>EX.MET_SOMATIC_VARIANT_BURDEN</t>
+  </si>
+  <si>
+    <t>snv_burden.value</t>
   </si>
 </sst>
 </file>
@@ -1096,10 +1096,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1123,7 +1123,7 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K2" t="s">
         <v>17</v>
@@ -1131,10 +1131,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -1158,18 +1158,18 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -1193,10 +1193,10 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1204,7 +1204,7 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K5" t="s">
         <v>16</v>
@@ -1239,7 +1239,7 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1263,10 +1263,10 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1274,7 +1274,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1298,10 +1298,10 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1309,7 +1309,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1333,10 +1333,10 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="K8" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1344,7 +1344,7 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1364,10 +1364,10 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="K9" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>